<commit_message>
Applied some beautification to make app pleasant without interferering with the functionalities of the application
</commit_message>
<xml_diff>
--- a/Bug Fix Log Bits CodeForge.xlsx
+++ b/Bug Fix Log Bits CodeForge.xlsx
@@ -1,9 +1,9 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30516"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30524"/>
   <workbookPr defaultThemeVersion="166925"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{62DB66E3-B423-4A56-9706-D786A421FC85}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{7E1829DC-D208-4EED-AB94-76093B9FA89E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="41">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="36">
   <si>
     <t>#</t>
   </si>
@@ -52,21 +52,6 @@
   </si>
   <si>
     <t>How You Tested the Fix</t>
-  </si>
-  <si>
-    <t>Course list duplicates after uploading another file</t>
-  </si>
-  <si>
-    <t>Uploaded two Excel files sequentially</t>
-  </si>
-  <si>
-    <t>Existing course options were not cleared</t>
-  </si>
-  <si>
-    <t>Cleared existing options before adding new courses</t>
-  </si>
-  <si>
-    <t>Uploaded 2 files and verified unique course list</t>
   </si>
   <si>
     <t>Average shows an incorrect value when no students are present</t>
@@ -564,14 +549,15 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F8"/>
+  <dimension ref="A1:F7"/>
   <sheetFormatPr defaultColWidth="25.7109375" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="9.28515625" style="4" customWidth="1"/>
-    <col min="2" max="16384" width="25.7109375" style="4"/>
+    <col min="2" max="6" width="35.7109375" style="4" customWidth="1"/>
+    <col min="7" max="16384" width="25.7109375" style="4"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" s="2" customFormat="1" ht="36">
+    <row r="1" spans="1:6" s="2" customFormat="1" ht="17.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -591,7 +577,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:6" ht="53.25">
+    <row r="2" spans="1:6" ht="36">
       <c r="A2" s="3">
         <v>1</v>
       </c>
@@ -611,7 +597,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="3" spans="1:6" ht="53.25">
+    <row r="3" spans="1:6" ht="105.75">
       <c r="A3" s="3">
         <v>2</v>
       </c>
@@ -631,7 +617,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="4" spans="1:6" ht="141">
+    <row r="4" spans="1:6" ht="176.25">
       <c r="A4" s="3">
         <v>3</v>
       </c>
@@ -651,7 +637,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="5" spans="1:6" ht="246.75">
+    <row r="5" spans="1:6" ht="159">
       <c r="A5" s="3">
         <v>4</v>
       </c>
@@ -671,7 +657,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="6" spans="1:6" ht="246.75">
+    <row r="6" spans="1:6" ht="176.25">
       <c r="A6" s="3">
         <v>5</v>
       </c>
@@ -691,7 +677,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="7" spans="1:6" ht="282.75">
+    <row r="7" spans="1:6" ht="211.5">
       <c r="A7" s="3">
         <v>6</v>
       </c>
@@ -709,26 +695,6 @@
       </c>
       <c r="F7" s="3" t="s">
         <v>35</v>
-      </c>
-    </row>
-    <row r="8" spans="1:6" ht="282.75">
-      <c r="A8" s="3">
-        <v>7</v>
-      </c>
-      <c r="B8" s="3" t="s">
-        <v>36</v>
-      </c>
-      <c r="C8" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="D8" s="3" t="s">
-        <v>38</v>
-      </c>
-      <c r="E8" s="3" t="s">
-        <v>39</v>
-      </c>
-      <c r="F8" s="3" t="s">
-        <v>40</v>
       </c>
     </row>
   </sheetData>

</xml_diff>